<commit_message>
Revise site selection: $250 price cap + exclude just-built placements
- Cap every placement at <= $250 per site
- Add the user-supplied May-Aug '25 just-built placements to the exclusion
  set on top of Ahrefs + Semrush referring domains (not yet indexed)
- Result: 30 relevant, not-used sites (20 Core + 10 Additional),
  total placement cost ~$5,057, avg ~$168

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTSVFSSCJZESeLBYWra4gT
</commit_message>
<xml_diff>
--- a/BlueGoatCyber_Site_Selection.xlsx
+++ b/BlueGoatCyber_Site_Selection.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Site Selection'!$A$1:$L$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Site Selection'!$A$1:$L$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -180,10 +180,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -556,13 +556,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
@@ -641,7 +641,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>cybernews.com</t>
+          <t>hackmd.io</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -651,36 +651,36 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Cybersecurity</t>
+          <t>Cybersecurity/Dev</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Leading independent cybersecurity news &amp; research publication</t>
+          <t>Collaborative docs platform; dev &amp; security audience</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>Technology, Tech, Innovation, Cybersecurity, News</t>
+          <t>Business, Entrepreneurship, Cybersecurity</t>
         </is>
       </c>
       <c r="G2" s="7" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="J2" s="8" t="n">
-        <v>3416624</v>
+        <v>274538</v>
       </c>
       <c r="K2" s="8" t="n">
-        <v>39175</v>
+        <v>86693</v>
       </c>
       <c r="L2" s="9" t="n">
-        <v>582</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3">
@@ -689,7 +689,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>cybersecuritynews.com</t>
+          <t>globalcybersecuritynetwork.com</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -704,31 +704,31 @@
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>Dedicated cybersecurity news (breaches, threats, vulns)</t>
+          <t>Cybersecurity companies directory, news &amp; careers</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>Android, Apple, Attack, Breaches, Cisco, Cloud, Cyber, Cyber Attack, Cybersecurity, Cyversecurity, Data, Data Privacy, Day, English, Firewall, Google, Hacking, Hacks, Industry Market, IS, News, Other, Scientific Reporting, Tech, Technology, Threats, Top, Training, Vulnerability, What, Zero</t>
+          <t>English: Technology, Cybersecurity, Careers, Education, Events, Business</t>
         </is>
       </c>
       <c r="G3" s="14" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="I3" s="14" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="J3" s="15" t="n">
-        <v>37424</v>
+        <v>5584</v>
       </c>
       <c r="K3" s="15" t="n">
-        <v>11344</v>
+        <v>1451</v>
       </c>
       <c r="L3" s="16" t="n">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4">
@@ -737,7 +737,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>hackread.com</t>
+          <t>devopsschool.com</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -747,36 +747,36 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Cybersecurity</t>
+          <t>Cybersecurity/Dev</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Infosec / hacking &amp; security news outlet</t>
+          <t>DevOps / DevSecOps training &amp; tutorials</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>News &amp; Media, Media, Journalism, Cybersecurity</t>
+          <t>Technology, Education, DevOps, Training</t>
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>23140</v>
+        <v>30028</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>13532</v>
+        <v>3664</v>
       </c>
       <c r="L4" s="9" t="n">
-        <v>256</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5">
@@ -785,7 +785,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>cybersecurityintelligence.com</t>
+          <t>invgate.com</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -795,36 +795,36 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Cybersecurity</t>
+          <t>IT/Security</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Cyber threat-intelligence directory &amp; news</t>
+          <t>ITSM &amp; IT management platform blog (security-adjacent)</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>English: Cybersecurity News, Threat Intelligence, Industry Insights</t>
+          <t>Business Solutions, IT Management, Software, Customer Service</t>
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="J5" s="15" t="n">
-        <v>30513</v>
+        <v>265910</v>
       </c>
       <c r="K5" s="15" t="n">
-        <v>3104</v>
+        <v>4812</v>
       </c>
       <c r="L5" s="16" t="n">
-        <v>450</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6">
@@ -833,7 +833,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>cm-alliance.com</t>
+          <t>sqlservercentral.com</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -841,38 +841,38 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Cybersecurity</t>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>IT/Dev</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Cyber Management Alliance – incident response &amp; training</t>
+          <t>SQL Server / database admin community (data security)</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>English: Technology, Cybersecurity, Business, Education</t>
+          <t>English: SQL Server, Database Administration, Database Development, T-SQL, Business Intelligence, Azure SQL, Performance, Tutorials, Community</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>19408</v>
+        <v>89551</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>3582</v>
+        <v>31848</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>695</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -881,7 +881,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>fastestvpn.com</t>
+          <t>dev.to</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -889,38 +889,38 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Cybersecurity</t>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Software/Dev</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Security/VPN &amp; privacy blog</t>
+          <t>Large developer community (programming, security)</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>App, Blogs, CBD, Cybersecurity, English, Protect, Secure Email, Server, Tech, VPN, VPN Resources</t>
+          <t>English: Technology, Programming, Coding, Community</t>
         </is>
       </c>
       <c r="G7" s="14" t="n">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="I7" s="14" t="n">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="J7" s="15" t="n">
-        <v>452098</v>
+        <v>2011489</v>
       </c>
       <c r="K7" s="15" t="n">
-        <v>13689</v>
+        <v>123886</v>
       </c>
       <c r="L7" s="16" t="n">
-        <v>660</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
@@ -929,7 +929,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>cyberpanel.net</t>
+          <t>analyticsinsight.net</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -937,38 +937,38 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>Software/Security</t>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Web-hosting control panel; security &amp; tech audience</t>
+          <t>AI, data science &amp; emerging-tech publication</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>English: Technology, Web Hosting, Software, Business</t>
+          <t>Analytics, Data Science, Technology, Business Intelligence</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>30721</v>
+        <v>112033</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>35935</v>
+        <v>30574</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>450</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9">
@@ -977,7 +977,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>hackmd.io</t>
+          <t>educba.com</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -985,38 +985,38 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Software/Dev</t>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Collaborative docs platform; dev/security audience</t>
+          <t>Tech education &amp; online-courses publisher</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Business, Entrepreneurship, Cybersecurity</t>
+          <t>English: Online Courses, Education, Technology, Business</t>
         </is>
       </c>
       <c r="G9" s="14" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="J9" s="15" t="n">
-        <v>274538</v>
+        <v>164489</v>
       </c>
       <c r="K9" s="15" t="n">
-        <v>86693</v>
+        <v>22421</v>
       </c>
       <c r="L9" s="16" t="n">
-        <v>61</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>dev.to</t>
+          <t>techimply.com</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1040,31 +1040,31 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Large developer community (programming, security)</t>
+          <t>Software discovery &amp; web-development content</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>English: Technology, Programming, Coding, Community</t>
+          <t>Web Development, Technology</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>2011489</v>
+        <v>28065</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>123886</v>
+        <v>4955</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>70</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>freecodecamp.org</t>
+          <t>rswebsols.com</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1088,31 +1088,31 @@
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Major programming &amp; tech education platform</t>
+          <t>Web development &amp; digital-services blog</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>English: Education, Technology, Programming</t>
+          <t>English: Web Development &amp; Digital Services, Web Design, SEO &amp; Hosting</t>
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J11" s="15" t="n">
-        <v>2428426</v>
+        <v>63175</v>
       </c>
       <c r="K11" s="15" t="n">
-        <v>70630</v>
+        <v>4364</v>
       </c>
       <c r="L11" s="16" t="n">
-        <v>775</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>researchgate.net</t>
+          <t>electronicsforu.com</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1131,36 +1131,36 @@
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Science/Tech</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Science &amp; technology research network (very high authority)</t>
+          <t>Electronics &amp; technology news</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>English: Education, Science, Technology</t>
+          <t>Electronics, DIY Projects, Technology News, Innovations</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>84</v>
+        <v>35</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>26471287</v>
+        <v>125324</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>805149</v>
+        <v>8465</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>400</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>cooltechzone.com</t>
+          <t>root-nation.com</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1184,31 +1184,31 @@
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Tech &amp; cybersecurity news/reviews</t>
+          <t>Technology, gadgets &amp; reviews</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>News &amp; Media, Media, Journalism, Tech News</t>
+          <t>Technology, Gadgets, Reviews</t>
         </is>
       </c>
       <c r="G13" s="14" t="n">
+        <v>41</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>29</v>
+      </c>
+      <c r="I13" s="14" t="n">
         <v>47</v>
       </c>
-      <c r="H13" s="14" t="n">
-        <v>59</v>
-      </c>
-      <c r="I13" s="14" t="n">
-        <v>53</v>
-      </c>
       <c r="J13" s="15" t="n">
-        <v>59600</v>
+        <v>42499</v>
       </c>
       <c r="K13" s="15" t="n">
-        <v>6404</v>
+        <v>6592</v>
       </c>
       <c r="L13" s="16" t="n">
-        <v>598</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>mspoweruser.com</t>
+          <t>propakistani.pk</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1232,31 +1232,31 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Microsoft/tech news site</t>
+          <t>Tech, telecom &amp; startups (geo diversity)</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>English: Technology, News, Business</t>
+          <t>Technology, Telecom, Business, Startups, News, Lifestyle</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>21454</v>
+        <v>600357</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>26422</v>
+        <v>23405</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>700</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>gagadget.com</t>
+          <t>danetsoft.com</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1280,31 +1280,31 @@
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Technology &amp; gadgets news</t>
+          <t>Technology, business &amp; marketing</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>Ukrainian: Technology, Gadgets, Science, News</t>
+          <t>English: Technology, Business, Marketing</t>
         </is>
       </c>
       <c r="G15" s="14" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="J15" s="15" t="n">
-        <v>28050</v>
+        <v>73165</v>
       </c>
       <c r="K15" s="15" t="n">
-        <v>13374</v>
+        <v>6016</v>
       </c>
       <c r="L15" s="16" t="n">
-        <v>734</v>
+        <v>190</v>
       </c>
     </row>
     <row r="16">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>analyticsinsight.net</t>
+          <t>fileion.com</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1328,31 +1328,31 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>AI, data science &amp; emerging-tech publication</t>
+          <t>Software &amp; technology site</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Analytics, Data Science, Technology, Business Intelligence</t>
+          <t>Technology, Tech, Innovation</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J16" s="8" t="n">
-        <v>112033</v>
+        <v>603439</v>
       </c>
       <c r="K16" s="8" t="n">
-        <v>30574</v>
+        <v>1864</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>250</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>livemint.com</t>
+          <t>hardreset.info</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1369,38 +1369,38 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
-        <is>
-          <t>News/Business</t>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Major business &amp; market news (high authority)</t>
+          <t>Devices, gadgets &amp; how-to tech</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>English: Business &amp; Market News, Companies, Markets, Technology, Money, Mutual Funds, Insurance, Auto, Industry, Personal Finance, Opinion</t>
+          <t>Computers, Gadgets, Hardware, Laptops, SEO, Smartphones, Software, Technology, Tutorials, Digital, IT, Learning, Innovation</t>
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>80</v>
+        <v>46</v>
       </c>
       <c r="H17" s="14" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="J17" s="15" t="n">
-        <v>11342474</v>
+        <v>298233</v>
       </c>
       <c r="K17" s="15" t="n">
-        <v>126740</v>
+        <v>14413</v>
       </c>
       <c r="L17" s="16" t="n">
-        <v>560</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>business-standard.com</t>
+          <t>barchart.com</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1417,38 +1417,38 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="D18" s="22" t="inlineStr">
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>News/Business</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Leading business/financial news daily</t>
+          <t>Markets, finance &amp; data platform (high authority)</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>News, Culture, Markets, Politics, Banking &amp; Finance, Education, Politics, Technology &amp; Gadgets, News &amp; Media, Business &amp; Finance, General</t>
+          <t>Business, Finance, Markets, Investing, Economy, Technology, Crypto, Trading, Personal Finance</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>4686795</v>
+        <v>3996423</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>109648</v>
+        <v>32405</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>380</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19">
@@ -1465,7 +1465,7 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="22" t="inlineStr">
         <is>
           <t>News/Business</t>
         </is>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>modernghana.com</t>
+          <t>zeebiz.com</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1513,38 +1513,38 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="D20" s="22" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>News/Business</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>General news/business – geographic diversity</t>
+          <t>Business &amp; stock-market news</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>English: News, Politics, Business</t>
+          <t>English: Business News, Stock Market, Finance, Markets, Sectors, Tax</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>559184</v>
+        <v>1235300</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>20107</v>
+        <v>29525</v>
       </c>
       <c r="L20" s="9" t="n">
-        <v>610</v>
+        <v>240</v>
       </c>
     </row>
     <row r="21">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>biospace.com</t>
+          <t>japantimes.co.jp</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1561,38 +1561,38 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
-        <is>
-          <t>Health/MedTech</t>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>News/Business</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>Biotech &amp; pharma news – fits medical-device security niche</t>
+          <t>Major news outlet – business/tech (geo diversity)</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>English: Biotechnology, Pharmaceuticals, Clinical Research, Business, Careers</t>
+          <t>English: News, Japan, Politics, Business, Culture</t>
         </is>
       </c>
       <c r="G21" s="14" t="n">
+        <v>57</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>48</v>
+      </c>
+      <c r="I21" s="14" t="n">
         <v>49</v>
       </c>
-      <c r="H21" s="14" t="n">
-        <v>63</v>
-      </c>
-      <c r="I21" s="14" t="n">
-        <v>57</v>
-      </c>
       <c r="J21" s="15" t="n">
-        <v>92436</v>
+        <v>519483</v>
       </c>
       <c r="K21" s="15" t="n">
-        <v>29719</v>
+        <v>106974</v>
       </c>
       <c r="L21" s="16" t="n">
-        <v>805</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>webcampus.unr.edu</t>
+          <t>bbntimes.com</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -1609,35 +1609,35 @@
           <t>Additional</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>Science/Tech</t>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>News/Business</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>.edu (Univ. of Nevada) – high-trust education/tech domain</t>
+          <t>Business, technology &amp; economy magazine</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>English: Education, Technology</t>
+          <t>Business, Technology, Economy, Finance</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>870128</v>
+        <v>537885</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>1172</v>
+        <v>12395</v>
       </c>
       <c r="L22" s="9" t="n">
         <v>250</v>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>osnews.com</t>
+          <t>thesiliconreview.com</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -1657,38 +1657,38 @@
           <t>Additional</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Software/Dev</t>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>News/Business</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>Long-running technology &amp; software news site</t>
+          <t>Business &amp; technology magazine</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>English: Technology, Software, News</t>
+          <t>Business, Energyresources, English, Finance, Games, Industry, Leadership, Leadershipguide, Magazine, News, Reviews, Socialmedia, Startup, Tech</t>
         </is>
       </c>
       <c r="G23" s="14" t="n">
         <v>39</v>
       </c>
       <c r="H23" s="14" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="I23" s="14" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="J23" s="15" t="n">
-        <v>12102</v>
+        <v>11962</v>
       </c>
       <c r="K23" s="15" t="n">
-        <v>12508</v>
+        <v>6293</v>
       </c>
       <c r="L23" s="16" t="n">
-        <v>760</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>tuaw.com</t>
+          <t>stockhouse.com</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1705,38 +1705,38 @@
           <t>Additional</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
-        <is>
-          <t>Technology</t>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>News/Business</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Apple / consumer-tech reviews &amp; news</t>
+          <t>Finance &amp; stock-market community</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>English: Apple, Technology, Reviews, How-To Guides</t>
+          <t>Finance, Stock Market, Canada</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="J24" s="8" t="n">
-        <v>143852</v>
+        <v>170157</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>16708</v>
+        <v>19403</v>
       </c>
       <c r="L24" s="9" t="n">
-        <v>400</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>phandroid.com</t>
+          <t>homebusinessmag.com</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -1753,38 +1753,38 @@
           <t>Additional</t>
         </is>
       </c>
-      <c r="D25" s="20" t="inlineStr">
-        <is>
-          <t>Technology</t>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>News/Business</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>Android &amp; mobile-tech news</t>
+          <t>Home-business &amp; entrepreneurship magazine</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>Android, Android, Apps, Carriers, Deals, English, Forums, Games, Mobile, Mobile Apps, Mobile Phones, News, OS Guide, Phones, Reviews, Tablets, Tech</t>
+          <t>Business, Home-Based, Magazine</t>
         </is>
       </c>
       <c r="G25" s="14" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H25" s="14" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="I25" s="14" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="J25" s="15" t="n">
-        <v>45668</v>
+        <v>34365</v>
       </c>
       <c r="K25" s="15" t="n">
-        <v>17976</v>
+        <v>8730</v>
       </c>
       <c r="L25" s="16" t="n">
-        <v>510</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>spacedaily.com</t>
+          <t>webcampus.unr.edu</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -1803,36 +1803,36 @@
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Science/Tech</t>
+          <t>Science/Edu</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Space, science &amp; technology news</t>
+          <t>.edu (Univ. of Nevada) – high-trust education/tech</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>English: Space, Science, Astronomy, Technology</t>
+          <t>English: Education, Technology</t>
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="H26" s="7" t="n">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>90533</v>
+        <v>870128</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>15494</v>
+        <v>1172</v>
       </c>
       <c r="L26" s="9" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
     </row>
     <row r="27">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>designrush.com</t>
+          <t>essex.ac.uk</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
@@ -1851,36 +1851,36 @@
       </c>
       <c r="D27" s="20" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Science/Edu</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>B2B agency directory – web/app dev, SEO, fintech</t>
+          <t>.ac.uk (University of Essex) – high-trust academic</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr">
         <is>
-          <t>Web Design, SEO, App Development, Fintech</t>
+          <t>English: Higher education, Undergraduate &amp; postgraduate courses, Social sciences &amp; health studies</t>
         </is>
       </c>
       <c r="G27" s="14" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="H27" s="14" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="I27" s="14" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="J27" s="15" t="n">
-        <v>399467</v>
+        <v>333806</v>
       </c>
       <c r="K27" s="15" t="n">
-        <v>42381</v>
+        <v>26009</v>
       </c>
       <c r="L27" s="16" t="n">
-        <v>820</v>
+        <v>250</v>
       </c>
     </row>
     <row r="28">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>ruby-doc.org</t>
+          <t>spacedaily.com</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -1897,38 +1897,38 @@
           <t>Additional</t>
         </is>
       </c>
-      <c r="D28" s="17" t="inlineStr">
-        <is>
-          <t>Software/Dev</t>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>Science/Tech</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Ruby developer documentation &amp; tech audience</t>
+          <t>Space, science &amp; technology news</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>Technology, Tech, Innovation</t>
+          <t>English: Space, Science, Astronomy, Technology</t>
         </is>
       </c>
       <c r="G28" s="7" t="n">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H28" s="7" t="n">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>183727</v>
+        <v>90533</v>
       </c>
       <c r="K28" s="8" t="n">
-        <v>10384</v>
+        <v>15494</v>
       </c>
       <c r="L28" s="9" t="n">
-        <v>316</v>
+        <v>240</v>
       </c>
     </row>
     <row r="29">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>hostpapa.com</t>
+          <t>medindia.net</t>
         </is>
       </c>
       <c r="C29" s="14" t="inlineStr">
@@ -1945,38 +1945,38 @@
           <t>Additional</t>
         </is>
       </c>
-      <c r="D29" s="18" t="inlineStr">
-        <is>
-          <t>Software/Security</t>
+      <c r="D29" s="23" t="inlineStr">
+        <is>
+          <t>Health/MedTech</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>Web hosting &amp; domain security services</t>
+          <t>Medical &amp; health information (fits med-device niche)</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>English: Web hosting services, Domain registration, Small business online solutions, Cloud hosting</t>
+          <t>English: Health, Wellness, Medical Information</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="H29" s="14" t="n">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="I29" s="14" t="n">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="J29" s="15" t="n">
-        <v>23503</v>
+        <v>613038</v>
       </c>
       <c r="K29" s="15" t="n">
-        <v>36204</v>
+        <v>19125</v>
       </c>
       <c r="L29" s="16" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
     </row>
     <row r="30">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>hostadvice.com</t>
+          <t>techylist.com</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -2000,31 +2000,31 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Hosting &amp; tech reviews platform</t>
+          <t>Technology, apps &amp; how-to</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>English: Technology, Business, Education</t>
+          <t>English: Technology, Apps, Downloads, How-To</t>
         </is>
       </c>
       <c r="G30" s="7" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="J30" s="8" t="n">
-        <v>91111</v>
+        <v>3645809</v>
       </c>
       <c r="K30" s="8" t="n">
-        <v>8807</v>
+        <v>8278</v>
       </c>
       <c r="L30" s="9" t="n">
-        <v>780</v>
+        <v>250</v>
       </c>
     </row>
     <row r="31">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>drwindows.de</t>
+          <t>getassist.net</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
@@ -2041,282 +2041,42 @@
           <t>Additional</t>
         </is>
       </c>
-      <c r="D31" s="18" t="inlineStr">
-        <is>
-          <t>Software/Dev</t>
+      <c r="D31" s="20" t="inlineStr">
+        <is>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>Windows/Microsoft tech community (DE)</t>
+          <t>Technology, business tools &amp; tips</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr">
         <is>
-          <t>German: Technology, Microsoft, Software, Windows</t>
+          <t>English: Technology, Business, Tools, Internet, Marketing, Online Services</t>
         </is>
       </c>
       <c r="G31" s="14" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H31" s="14" t="n">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="I31" s="14" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="J31" s="15" t="n">
-        <v>72455</v>
+        <v>131381</v>
       </c>
       <c r="K31" s="15" t="n">
-        <v>6164</v>
+        <v>4292</v>
       </c>
       <c r="L31" s="16" t="n">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>barchart.com</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Additional</t>
-        </is>
-      </c>
-      <c r="D32" s="22" t="inlineStr">
-        <is>
-          <t>News/Business</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Markets, finance &amp; data platform (high authority)</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>Business, Finance, Markets, Investing, Economy, Technology, Crypto, Trading, Personal Finance</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="n">
-        <v>68</v>
-      </c>
-      <c r="H32" s="7" t="n">
-        <v>52</v>
-      </c>
-      <c r="I32" s="7" t="n">
-        <v>51</v>
-      </c>
-      <c r="J32" s="8" t="n">
-        <v>3996423</v>
-      </c>
-      <c r="K32" s="8" t="n">
-        <v>32405</v>
-      </c>
-      <c r="L32" s="9" t="n">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>advfn.com</t>
-        </is>
-      </c>
-      <c r="C33" s="14" t="inlineStr">
-        <is>
-          <t>Additional</t>
-        </is>
-      </c>
-      <c r="D33" s="21" t="inlineStr">
-        <is>
-          <t>News/Business</t>
-        </is>
-      </c>
-      <c r="E33" s="13" t="inlineStr">
-        <is>
-          <t>Financial markets &amp; investing news</t>
-        </is>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>Finance, Stocks, Investments, Market News</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="n">
-        <v>66</v>
-      </c>
-      <c r="H33" s="14" t="n">
-        <v>48</v>
-      </c>
-      <c r="I33" s="14" t="n">
-        <v>44</v>
-      </c>
-      <c r="J33" s="15" t="n">
-        <v>3379549</v>
-      </c>
-      <c r="K33" s="15" t="n">
-        <v>26308</v>
-      </c>
-      <c r="L33" s="16" t="n">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>fxstreet.com</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Additional</t>
-        </is>
-      </c>
-      <c r="D34" s="22" t="inlineStr">
-        <is>
-          <t>News/Business</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>Finance / markets analysis publication</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>Finance, Forex, Trading, Analysis</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="n">
-        <v>63</v>
-      </c>
-      <c r="H34" s="7" t="n">
-        <v>51</v>
-      </c>
-      <c r="I34" s="7" t="n">
-        <v>53</v>
-      </c>
-      <c r="J34" s="8" t="n">
-        <v>1412127</v>
-      </c>
-      <c r="K34" s="8" t="n">
-        <v>31467</v>
-      </c>
-      <c r="L34" s="9" t="n">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>biz.liga.net</t>
-        </is>
-      </c>
-      <c r="C35" s="14" t="inlineStr">
-        <is>
-          <t>Additional</t>
-        </is>
-      </c>
-      <c r="D35" s="21" t="inlineStr">
-        <is>
-          <t>News/Business</t>
-        </is>
-      </c>
-      <c r="E35" s="13" t="inlineStr">
-        <is>
-          <t>Ukrainian business &amp; technology news (AS67)</t>
-        </is>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>Ukrainian: Business, Finance, Technology, Real Estate, Automotive, News</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="n">
-        <v>67</v>
-      </c>
-      <c r="H35" s="14" t="n">
-        <v>27</v>
-      </c>
-      <c r="I35" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="J35" s="15" t="n">
-        <v>1458660</v>
-      </c>
-      <c r="K35" s="15" t="n">
-        <v>7051</v>
-      </c>
-      <c r="L35" s="16" t="n">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>sfexaminer.com</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>Additional</t>
-        </is>
-      </c>
-      <c r="D36" s="22" t="inlineStr">
-        <is>
-          <t>News/Business</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>US news outlet with technology/business coverage</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>English: News, Politics, Technology, Business, Urban Development, Climate</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="n">
-        <v>46</v>
-      </c>
-      <c r="H36" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="I36" s="7" t="n">
-        <v>47</v>
-      </c>
-      <c r="J36" s="8" t="n">
-        <v>53583</v>
-      </c>
-      <c r="K36" s="8" t="n">
-        <v>33314</v>
-      </c>
-      <c r="L36" s="9" t="n">
-        <v>650</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L36"/>
+  <autoFilter ref="A1:L31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2327,7 +2087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2336,21 +2096,21 @@
     <row r="1">
       <c r="A1" s="24" t="inlineStr">
         <is>
-          <t>Site Selection – Blue Goat Cyber (bluegoatcyber.com)</t>
+          <t>Site Selection - Blue Goat Cyber (bluegoatcyber.com)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>35 guest-post / placement targets selected from the Reachgorilla inventory (13,405 sites).</t>
+          <t>30 guest-post / placement targets from the Reachgorilla inventory (13,405 sites).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tier 'Core' = top 20 recommended; 'Additional' = 15 further strong, on-topic options.</t>
+          <t>Tier 'Core' = top 20 recommended; 'Additional' = further strong, on-topic options.</t>
         </is>
       </c>
     </row>
@@ -2367,28 +2127,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Relevance to a cybersecurity / penetration-testing / medical-device-security company</t>
+          <t xml:space="preserve">  - Relevance to a cybersecurity / pen-testing / medical-device-security company</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Requested mix: cybersecurity-niche + technology + developer + news/business sites</t>
+          <t xml:space="preserve">  - Mix of cybersecurity/IT-security, technology, developer and news/business sites</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Quality gate: Authority Score (AS) &gt;= ~36, Trust Flow (TF) &gt;= ~22, real organic traffic</t>
+          <t xml:space="preserve">  - Quality gate: Authority Score (AS) &gt;= ~35, Trust Flow (TF) &gt;= ~20, real organic traffic</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Actionable price band (kept &lt;= ~$900 per placement)</t>
+          <t xml:space="preserve">  - PRICE CAP: every site is &lt;= $250 per placement</t>
         </is>
       </c>
     </row>
@@ -2405,52 +2165,90 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Cross-referenced against Blue Goat Cyber's live backlink profile using BOTH Ahrefs and Semrush.</t>
+          <t xml:space="preserve">  - Existing referring domains pulled from BOTH Ahrefs and Semrush; any domain already</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Any domain already linking to bluegoatcyber.com in EITHER tool was removed.</t>
+          <t xml:space="preserve">    linking to bluegoatcyber.com in either tool was removed.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Examples removed as already-used: linuxsecurity.com, securityboulevard.com, gbhackers.com,</t>
+          <t xml:space="preserve">  - PLUS just-built placements you supplied (May-Aug '25) that are not yet indexed, e.g.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cyberkendra.com, businessinsider.com, crunchbase.com, indiehackers.com, techbullion.com,</t>
+          <t xml:space="preserve">    cyberpress.org, cybersecuritynews.com, cyberkendra.com, cybersecurityintelligence.com,</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">    iemlabs.com, opsmatters.com, velog.io, coruzant.com, theenterpriseworld.com, hashnode.dev.</t>
+          <t xml:space="preserve">    opsmatters.com, linuxsecurity.com, hackread.com, gbhackers.com, hacker9.com,</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    securitysenses.com, guardiandigital.com, winbuzzer.com, codeitbro.com, medigy.com,</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Metric key: AS = Authority Score | TF = Trust Flow | CF = Citation Flow |</t>
+          <t xml:space="preserve">    technology.org, openmedscience.com, and the rest of your May-Aug list.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>RD = Referring Domains | Traffic = est. monthly organic | Price = listed placement cost.</t>
+      <c r="A19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>Note: under the $250 cap most pure-cyber publications are now either already used or</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>above budget (e.g. cybernews $582, cm-alliance $695, fastestvpn $660, cyberpanel $450),</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>so this list leans into tech / dev / IT-security / news-business, as you okayed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Metric key: AS=Authority Score | TF=Trust Flow | CF=Citation Flow | RD=Referring Domains |</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Traffic=est. monthly organic | Price=listed placement cost.</t>
         </is>
       </c>
     </row>

</xml_diff>